<commit_message>
Update reviewed Core200 tasks
</commit_message>
<xml_diff>
--- a/tasks/cross_device/linux_android_assets/linux_android_1185/source/tmp/meetings/attendees.xlsx
+++ b/tasks/cross_device/linux_android_assets/linux_android_1185/source/tmp/meetings/attendees.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,6 +437,11 @@
           <t>status</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>phone</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -459,6 +464,11 @@
           <t>attend</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>5551201185</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -481,6 +491,11 @@
           <t>attend</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>5551201186</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -501,6 +516,11 @@
       <c r="D4" t="inlineStr">
         <is>
           <t>archived</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>5551201195</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Sync complete Core200 task bundle
</commit_message>
<xml_diff>
--- a/tasks/cross_device/linux_android_assets/linux_android_1185/source/tmp/meetings/attendees.xlsx
+++ b/tasks/cross_device/linux_android_assets/linux_android_1185/source/tmp/meetings/attendees.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>5551201185</t>
+          <t>5557312</t>
         </is>
       </c>
     </row>
@@ -493,7 +493,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>5551201186</t>
+          <t>5558426</t>
         </is>
       </c>
     </row>
@@ -520,7 +520,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>5551201195</t>
+          <t>5559047</t>
         </is>
       </c>
     </row>

</xml_diff>